<commit_message>
fix(gui-beta-r1): WP-H W12 PopulationStage 原生风格标签着色（去 contentItem 覆盖，真机 0 告警）
- src/ui/gui/qml/stages/PopulationStage.qml：移除 RadioButton 的 contentItem 覆盖，
  改为 palette.windowText（含 disabled/inactive）着色 —— 消除 Windows 原生风格下
  「自定义 contentItem」运行期告警（627 行族，真机 107 条 → 0），净 −4 行。
- src/tests/test_gui/test_wph_w12_population_palette.py：新增 W12 标签调色断言（P-W12.1–4）。

验证：Owner 真机 V1 = PASS（contentItem / QML warning / ERROR = 0/0/0）；
      G5 focused = PASS（无条件）；全量回归 2618 passed / 14 skipped / 0 failed；
      W01–W11 无回退。
基线：parent = eaebf5c（WP-H 前序 candidate）。
排除：docs/MVP 0.9 …/EOR MVP 1.0 目标版本规划 V1.1.xlsx（ambient，非本次变更）。
</commit_message>
<xml_diff>
--- a/docs/MVP 0.9 项目管理/01_需求与版本规划/EOR MVP 1.0 目标版本规划 V1.1.xlsx
+++ b/docs/MVP 0.9 项目管理/01_需求与版本规划/EOR MVP 1.0 目标版本规划 V1.1.xlsx
@@ -1,10 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kerl\PycharmProjects\Eagle of Rome\docs\MVP 0.9 项目管理\01_需求与版本规划\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView windowHeight="17775" activeTab="1"/>
+    <workbookView windowHeight="17175" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="人物设定" sheetId="1" r:id="rId1"/>
@@ -3685,13 +3690,13 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="9"/>
       <color rgb="FF000000"/>
       <name val="Consolas"/>
       <charset val="134"/>
     </font>
     <font>
-      <sz val="9"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Consolas"/>
       <charset val="134"/>
@@ -4716,7 +4721,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1 1" defaultPivotStyle="PivotStylePreset2_Accent1 1">
-    <tableStyle name="TableStylePreset3_Accent1 1" pivot="0" count="7" xr9:uid="{02CC191A-CB85-447D-A12E-4AD26D929F4B}">
+    <tableStyle name="TableStylePreset3_Accent1 1" pivot="0" count="7" xr9:uid="{1C2B5C83-D2AA-4274-9722-D03BEF5E6166}">
       <tableStyleElement type="wholeTable" dxfId="7"/>
       <tableStyleElement type="headerRow" dxfId="6"/>
       <tableStyleElement type="totalRow" dxfId="5"/>
@@ -4725,7 +4730,7 @@
       <tableStyleElement type="firstRowStripe" dxfId="2"/>
       <tableStyleElement type="firstColumnStripe" dxfId="1"/>
     </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1 1" table="0" count="10" xr9:uid="{4C31328B-8DBA-47F9-B89D-1D92FC4E42C7}">
+    <tableStyle name="PivotStylePreset2_Accent1 1" table="0" count="10" xr9:uid="{1EEB2907-4066-4F3A-935F-32610018FF4E}">
       <tableStyleElement type="headerRow" dxfId="17"/>
       <tableStyleElement type="totalRow" dxfId="16"/>
       <tableStyleElement type="firstRowStripe" dxfId="15"/>

</xml_diff>

<commit_message>
chore(gui-beta-r1): 还原非任务 ambient xlsx（WP-H W12 candidate 排除）
</commit_message>
<xml_diff>
--- a/docs/MVP 0.9 项目管理/01_需求与版本规划/EOR MVP 1.0 目标版本规划 V1.1.xlsx
+++ b/docs/MVP 0.9 项目管理/01_需求与版本规划/EOR MVP 1.0 目标版本规划 V1.1.xlsx
@@ -1,15 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kerl\PycharmProjects\Eagle of Rome\docs\MVP 0.9 项目管理\01_需求与版本规划\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <bookViews>
-    <workbookView windowHeight="17175" activeTab="4"/>
+    <workbookView windowHeight="17775" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="人物设定" sheetId="1" r:id="rId1"/>
@@ -3690,13 +3685,13 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Consolas"/>
       <charset val="134"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="9"/>
       <color rgb="FF000000"/>
       <name val="Consolas"/>
       <charset val="134"/>
@@ -4721,7 +4716,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1 1" defaultPivotStyle="PivotStylePreset2_Accent1 1">
-    <tableStyle name="TableStylePreset3_Accent1 1" pivot="0" count="7" xr9:uid="{1C2B5C83-D2AA-4274-9722-D03BEF5E6166}">
+    <tableStyle name="TableStylePreset3_Accent1 1" pivot="0" count="7" xr9:uid="{02CC191A-CB85-447D-A12E-4AD26D929F4B}">
       <tableStyleElement type="wholeTable" dxfId="7"/>
       <tableStyleElement type="headerRow" dxfId="6"/>
       <tableStyleElement type="totalRow" dxfId="5"/>
@@ -4730,7 +4725,7 @@
       <tableStyleElement type="firstRowStripe" dxfId="2"/>
       <tableStyleElement type="firstColumnStripe" dxfId="1"/>
     </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1 1" table="0" count="10" xr9:uid="{1EEB2907-4066-4F3A-935F-32610018FF4E}">
+    <tableStyle name="PivotStylePreset2_Accent1 1" table="0" count="10" xr9:uid="{4C31328B-8DBA-47F9-B89D-1D92FC4E42C7}">
       <tableStyleElement type="headerRow" dxfId="17"/>
       <tableStyleElement type="totalRow" dxfId="16"/>
       <tableStyleElement type="firstRowStripe" dxfId="15"/>

</xml_diff>